<commit_message>
Update fee collection and reports with latest transactions
Added new fee collection records and updated payment statuses in multiple CSV and Excel files to reflect recent transactions for November 2025. Adjusted 'Total_Fee_Paid' and 'Total_Due' fields for several students in fees_collection.csv. Updated Power BI dashboard and related reports to include the latest data.
</commit_message>
<xml_diff>
--- a/output_data/atom_report.xlsx
+++ b/output_data/atom_report.xlsx
@@ -21778,7 +21778,7 @@
       </c>
       <c r="M59" t="inlineStr">
         <is>
-          <t>NRNS</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="N59" t="inlineStr">
@@ -21803,7 +21803,7 @@
       </c>
       <c r="R59" t="inlineStr">
         <is>
-          <t/>
+          <t>14-Nov-2025 00:00:00</t>
         </is>
       </c>
       <c r="S59" t="inlineStr">
@@ -21878,12 +21878,12 @@
       </c>
       <c r="AG59" t="inlineStr">
         <is>
-          <t/>
+          <t>5</t>
         </is>
       </c>
       <c r="AH59" t="inlineStr">
         <is>
-          <t/>
+          <t>0.9</t>
         </is>
       </c>
       <c r="AI59" t="inlineStr">
@@ -21898,17 +21898,17 @@
       </c>
       <c r="AK59" t="inlineStr">
         <is>
-          <t/>
+          <t>5.9</t>
         </is>
       </c>
       <c r="AL59" t="inlineStr">
         <is>
-          <t/>
+          <t>7750.0</t>
         </is>
       </c>
       <c r="AM59" t="inlineStr">
         <is>
-          <t/>
+          <t>14-Nov-2025 00:00:00</t>
         </is>
       </c>
       <c r="AN59" t="inlineStr">
@@ -22150,7 +22150,7 @@
       </c>
       <c r="M60" t="inlineStr">
         <is>
-          <t>NRNS</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="N60" t="inlineStr">
@@ -22175,7 +22175,7 @@
       </c>
       <c r="R60" t="inlineStr">
         <is>
-          <t/>
+          <t>14-Nov-2025 00:00:00</t>
         </is>
       </c>
       <c r="S60" t="inlineStr">
@@ -22250,12 +22250,12 @@
       </c>
       <c r="AG60" t="inlineStr">
         <is>
-          <t/>
+          <t>5</t>
         </is>
       </c>
       <c r="AH60" t="inlineStr">
         <is>
-          <t/>
+          <t>0.9</t>
         </is>
       </c>
       <c r="AI60" t="inlineStr">
@@ -22270,17 +22270,17 @@
       </c>
       <c r="AK60" t="inlineStr">
         <is>
-          <t/>
+          <t>5.9</t>
         </is>
       </c>
       <c r="AL60" t="inlineStr">
         <is>
-          <t/>
+          <t>6750.0</t>
         </is>
       </c>
       <c r="AM60" t="inlineStr">
         <is>
-          <t/>
+          <t>14-Nov-2025 00:00:00</t>
         </is>
       </c>
       <c r="AN60" t="inlineStr">
@@ -22522,7 +22522,7 @@
       </c>
       <c r="M61" t="inlineStr">
         <is>
-          <t>NRNS</t>
+          <t>RNS</t>
         </is>
       </c>
       <c r="N61" t="inlineStr">
@@ -22547,7 +22547,7 @@
       </c>
       <c r="R61" t="inlineStr">
         <is>
-          <t/>
+          <t>14-Nov-2025 00:00:00</t>
         </is>
       </c>
       <c r="S61" t="inlineStr">
@@ -22622,12 +22622,12 @@
       </c>
       <c r="AG61" t="inlineStr">
         <is>
-          <t/>
+          <t>5</t>
         </is>
       </c>
       <c r="AH61" t="inlineStr">
         <is>
-          <t/>
+          <t>0.9</t>
         </is>
       </c>
       <c r="AI61" t="inlineStr">
@@ -22642,17 +22642,17 @@
       </c>
       <c r="AK61" t="inlineStr">
         <is>
-          <t/>
+          <t>5.9</t>
         </is>
       </c>
       <c r="AL61" t="inlineStr">
         <is>
-          <t/>
+          <t>11250.0</t>
         </is>
       </c>
       <c r="AM61" t="inlineStr">
         <is>
-          <t/>
+          <t>14-Nov-2025 00:00:00</t>
         </is>
       </c>
       <c r="AN61" t="inlineStr">
@@ -22894,7 +22894,7 @@
       </c>
       <c r="M62" t="inlineStr">
         <is>
-          <t>NRNS</t>
+          <t>RNS</t>
         </is>
       </c>
       <c r="N62" t="inlineStr">
@@ -22994,12 +22994,12 @@
       </c>
       <c r="AG62" t="inlineStr">
         <is>
-          <t/>
+          <t>5</t>
         </is>
       </c>
       <c r="AH62" t="inlineStr">
         <is>
-          <t/>
+          <t>0.9</t>
         </is>
       </c>
       <c r="AI62" t="inlineStr">
@@ -23014,12 +23014,12 @@
       </c>
       <c r="AK62" t="inlineStr">
         <is>
-          <t/>
+          <t>5.9</t>
         </is>
       </c>
       <c r="AL62" t="inlineStr">
         <is>
-          <t/>
+          <t>11250.0</t>
         </is>
       </c>
       <c r="AM62" t="inlineStr">
@@ -23266,310 +23266,3286 @@
       </c>
       <c r="M63" t="inlineStr">
         <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="N63" t="inlineStr">
+        <is>
+          <t>108566739973</t>
+        </is>
+      </c>
+      <c r="O63" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P63" t="inlineStr">
+        <is>
+          <t>0899053000000002</t>
+        </is>
+      </c>
+      <c r="Q63" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="R63" t="inlineStr">
+        <is>
+          <t>14-Nov-2025 00:00:00</t>
+        </is>
+      </c>
+      <c r="S63" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="T63" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="U63" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="V63" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="W63" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="X63" t="inlineStr">
+        <is>
+          <t>JAHNAVI KOLASANI</t>
+        </is>
+      </c>
+      <c r="Y63" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="Z63" t="inlineStr">
+        <is>
+          <t>9347559040</t>
+        </is>
+      </c>
+      <c r="AA63" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AB63" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AC63" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AD63" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AE63" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AF63" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AG63" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AH63" t="inlineStr">
+        <is>
+          <t>0.9</t>
+        </is>
+      </c>
+      <c r="AI63" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="AJ63" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="AK63" t="inlineStr">
+        <is>
+          <t>5.9</t>
+        </is>
+      </c>
+      <c r="AL63" t="inlineStr">
+        <is>
+          <t>11250.0</t>
+        </is>
+      </c>
+      <c r="AM63" t="inlineStr">
+        <is>
+          <t>14-Nov-2025 00:00:00</t>
+        </is>
+      </c>
+      <c r="AN63" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AO63" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AP63" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AQ63" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AR63" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AS63" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AT63" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="AU63" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AV63" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AW63" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AX63" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AY63" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AZ63" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BA63" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="BB63" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BC63" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BD63" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="BE63" t="inlineStr">
+        <is>
+          <t>19295</t>
+        </is>
+      </c>
+      <c r="BF63" t="inlineStr">
+        <is>
+          <t>263081,264584</t>
+        </is>
+      </c>
+      <c r="BG63" t="inlineStr">
+        <is>
+          <t>2037,2044</t>
+        </is>
+      </c>
+      <c r="BH63" t="inlineStr">
+        <is>
+          <t>eleven thousand two hundred fifty</t>
+        </is>
+      </c>
+      <c r="BI63" t="inlineStr">
+        <is>
+          <t>15599</t>
+        </is>
+      </c>
+      <c r="BJ63" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BK63" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BL63" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BM63" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BN63" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BO63" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BP63" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BQ63" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BR63" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BS63" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BT63" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="BU63" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BV63" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>753702</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>1234</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>11000316697401</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>1763131313</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>8550.00</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>14-Nov-2025 20:15:44</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="M64" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="N64" t="inlineStr">
+        <is>
+          <t>108572296490</t>
+        </is>
+      </c>
+      <c r="O64" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P64" t="inlineStr">
+        <is>
+          <t>100000036600</t>
+        </is>
+      </c>
+      <c r="Q64" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="R64" t="inlineStr">
+        <is>
+          <t>15-Nov-2025 00:00:00</t>
+        </is>
+      </c>
+      <c r="S64" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="T64" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="U64" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="V64" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="W64" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="X64" t="inlineStr">
+        <is>
+          <t>KOLASANI SYAMANTH LAKSHMI VEER</t>
+        </is>
+      </c>
+      <c r="Y64" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="Z64" t="inlineStr">
+        <is>
+          <t>9849989564</t>
+        </is>
+      </c>
+      <c r="AA64" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AB64" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AC64" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AD64" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AE64" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AF64" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AG64" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AH64" t="inlineStr">
+        <is>
+          <t>0.9</t>
+        </is>
+      </c>
+      <c r="AI64" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="AJ64" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="AK64" t="inlineStr">
+        <is>
+          <t>5.9</t>
+        </is>
+      </c>
+      <c r="AL64" t="inlineStr">
+        <is>
+          <t>8550.0</t>
+        </is>
+      </c>
+      <c r="AM64" t="inlineStr">
+        <is>
+          <t>15-Nov-2025 00:00:00</t>
+        </is>
+      </c>
+      <c r="AN64" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AO64" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AP64" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AQ64" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AR64" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AS64" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AT64" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="AU64" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AV64" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AW64" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AX64" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AY64" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AZ64" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BA64" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="BB64" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="BC64" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BD64" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="BE64" t="inlineStr">
+        <is>
+          <t>18669</t>
+        </is>
+      </c>
+      <c r="BF64" t="inlineStr">
+        <is>
+          <t>262480,264030</t>
+        </is>
+      </c>
+      <c r="BG64" t="inlineStr">
+        <is>
+          <t>2037,2041</t>
+        </is>
+      </c>
+      <c r="BH64" t="inlineStr">
+        <is>
+          <t>eight thousand five hundred fifty</t>
+        </is>
+      </c>
+      <c r="BI64" t="inlineStr">
+        <is>
+          <t>16595</t>
+        </is>
+      </c>
+      <c r="BJ64" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BK64" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BL64" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BM64" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BN64" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BO64" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BP64" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BQ64" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BR64" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BS64" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BT64" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="BU64" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BV64" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>753702</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>1234</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>11000316700245</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>1763132856</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>8850.00</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>14-Nov-2025 20:40:21</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="M65" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="N65" t="inlineStr">
+        <is>
+          <t>108572419761</t>
+        </is>
+      </c>
+      <c r="O65" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P65" t="inlineStr">
+        <is>
+          <t>100000036600</t>
+        </is>
+      </c>
+      <c r="Q65" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="R65" t="inlineStr">
+        <is>
+          <t>15-Nov-2025 00:00:00</t>
+        </is>
+      </c>
+      <c r="S65" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="T65" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="U65" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="V65" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="W65" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="X65" t="inlineStr">
+        <is>
+          <t>DUVVU BHARGAVA SRI SAI</t>
+        </is>
+      </c>
+      <c r="Y65" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="Z65" t="inlineStr">
+        <is>
+          <t>9502247535</t>
+        </is>
+      </c>
+      <c r="AA65" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AB65" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AC65" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AD65" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AE65" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AF65" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AG65" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AH65" t="inlineStr">
+        <is>
+          <t>0.9</t>
+        </is>
+      </c>
+      <c r="AI65" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="AJ65" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="AK65" t="inlineStr">
+        <is>
+          <t>5.9</t>
+        </is>
+      </c>
+      <c r="AL65" t="inlineStr">
+        <is>
+          <t>8850.0</t>
+        </is>
+      </c>
+      <c r="AM65" t="inlineStr">
+        <is>
+          <t>15-Nov-2025 00:00:00</t>
+        </is>
+      </c>
+      <c r="AN65" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AO65" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AP65" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AQ65" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AR65" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AS65" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AT65" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="AU65" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AV65" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AW65" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AX65" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AY65" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AZ65" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BA65" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="BB65" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="BC65" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BD65" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="BE65" t="inlineStr">
+        <is>
+          <t>18964</t>
+        </is>
+      </c>
+      <c r="BF65" t="inlineStr">
+        <is>
+          <t>262817,264320</t>
+        </is>
+      </c>
+      <c r="BG65" t="inlineStr">
+        <is>
+          <t>2037,2042</t>
+        </is>
+      </c>
+      <c r="BH65" t="inlineStr">
+        <is>
+          <t>eight thousand eight hundred fifty</t>
+        </is>
+      </c>
+      <c r="BI65" t="inlineStr">
+        <is>
+          <t>16036</t>
+        </is>
+      </c>
+      <c r="BJ65" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BK65" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BL65" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BM65" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BN65" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BO65" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BP65" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BQ65" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BR65" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BS65" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BT65" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="BU65" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BV65" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>753702</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>1234</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>11000316701281</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>1763133080</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>8350.00</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>14-Nov-2025 20:43:12</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="M66" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="N66" t="inlineStr">
+        <is>
+          <t>108572433794</t>
+        </is>
+      </c>
+      <c r="O66" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P66" t="inlineStr">
+        <is>
+          <t>100000036600</t>
+        </is>
+      </c>
+      <c r="Q66" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="R66" t="inlineStr">
+        <is>
+          <t>15-Nov-2025 00:00:00</t>
+        </is>
+      </c>
+      <c r="S66" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="T66" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="U66" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="V66" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="W66" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="X66" t="inlineStr">
+        <is>
+          <t>DUVVU BHARGAVA SRI SAI</t>
+        </is>
+      </c>
+      <c r="Y66" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="Z66" t="inlineStr">
+        <is>
+          <t>9502247535</t>
+        </is>
+      </c>
+      <c r="AA66" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AB66" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AC66" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AD66" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AE66" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AF66" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AG66" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AH66" t="inlineStr">
+        <is>
+          <t>0.9</t>
+        </is>
+      </c>
+      <c r="AI66" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="AJ66" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="AK66" t="inlineStr">
+        <is>
+          <t>5.9</t>
+        </is>
+      </c>
+      <c r="AL66" t="inlineStr">
+        <is>
+          <t>8350.0</t>
+        </is>
+      </c>
+      <c r="AM66" t="inlineStr">
+        <is>
+          <t>15-Nov-2025 00:00:00</t>
+        </is>
+      </c>
+      <c r="AN66" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AO66" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AP66" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AQ66" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AR66" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AS66" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AT66" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="AU66" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AV66" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AW66" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AX66" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AY66" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AZ66" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BA66" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="BB66" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="BC66" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BD66" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="BE66" t="inlineStr">
+        <is>
+          <t>18964</t>
+        </is>
+      </c>
+      <c r="BF66" t="inlineStr">
+        <is>
+          <t>265970</t>
+        </is>
+      </c>
+      <c r="BG66" t="inlineStr">
+        <is>
+          <t>2050</t>
+        </is>
+      </c>
+      <c r="BH66" t="inlineStr">
+        <is>
+          <t>eight thousand three hundred fifty</t>
+        </is>
+      </c>
+      <c r="BI66" t="inlineStr">
+        <is>
+          <t>16036</t>
+        </is>
+      </c>
+      <c r="BJ66" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BK66" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BL66" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BM66" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BN66" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BO66" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BP66" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BQ66" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BR66" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BS66" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BT66" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="BU66" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BV66" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>753702</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>1234</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>11000316726912</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>1763173641</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>8850.00</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>15-Nov-2025 08:00:27</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="M67" t="inlineStr">
+        <is>
           <t>NRNS</t>
         </is>
       </c>
-      <c r="N63" t="inlineStr">
-        <is>
-          <t>108566739973</t>
-        </is>
-      </c>
-      <c r="O63" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="P63" t="inlineStr">
-        <is>
-          <t>0899053000000002</t>
-        </is>
-      </c>
-      <c r="Q63" t="inlineStr">
+      <c r="N67" t="inlineStr">
+        <is>
+          <t>108573859508</t>
+        </is>
+      </c>
+      <c r="O67" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P67" t="inlineStr">
+        <is>
+          <t>100000036600</t>
+        </is>
+      </c>
+      <c r="Q67" t="inlineStr">
         <is>
           <t>SIBL0000899</t>
         </is>
       </c>
-      <c r="R63" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="S63" t="inlineStr">
+      <c r="R67" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="S67" t="inlineStr">
         <is>
           <t>MERCHANT</t>
         </is>
       </c>
-      <c r="T63" t="inlineStr">
+      <c r="T67" t="inlineStr">
         <is>
           <t>UPI</t>
         </is>
       </c>
-      <c r="U63" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="V63" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="W63" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="X63" t="inlineStr">
-        <is>
-          <t>JAHNAVI KOLASANI</t>
-        </is>
-      </c>
-      <c r="Y63" t="inlineStr">
+      <c r="U67" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="V67" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="W67" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="X67" t="inlineStr">
+        <is>
+          <t>RASAJNA VOBBILISETTY</t>
+        </is>
+      </c>
+      <c r="Y67" t="inlineStr">
         <is>
           <t>kotakschoolvsp@gmail.com</t>
         </is>
       </c>
-      <c r="Z63" t="inlineStr">
-        <is>
-          <t>9347559040</t>
-        </is>
-      </c>
-      <c r="AA63" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="AB63" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="AC63" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="AD63" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="AE63" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="AF63" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="AG63" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="AH63" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="AI63" t="inlineStr">
+      <c r="Z67" t="inlineStr">
+        <is>
+          <t>9849969449</t>
+        </is>
+      </c>
+      <c r="AA67" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AB67" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AC67" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AD67" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AE67" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AF67" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AG67" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AH67" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AI67" t="inlineStr">
         <is>
           <t>0.00</t>
         </is>
       </c>
-      <c r="AJ63" t="inlineStr">
+      <c r="AJ67" t="inlineStr">
         <is>
           <t>0.00</t>
         </is>
       </c>
-      <c r="AK63" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="AL63" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="AM63" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="AN63" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="AO63" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="AP63" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="AQ63" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="AR63" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="AS63" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="AT63" t="inlineStr">
+      <c r="AK67" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AL67" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AM67" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AN67" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AO67" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AP67" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AQ67" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AR67" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AS67" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AT67" t="inlineStr">
         <is>
           <t>TRANSACTION IS SUCCESSFUL</t>
         </is>
       </c>
-      <c r="AU63" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="AV63" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="AW63" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="AX63" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="AY63" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="AZ63" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="BA63" t="inlineStr">
+      <c r="AU67" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AV67" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AW67" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AX67" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AY67" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AZ67" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BA67" t="inlineStr">
         <is>
           <t>UPI</t>
         </is>
       </c>
-      <c r="BB63" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="BC63" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="BD63" t="inlineStr">
+      <c r="BB67" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="BC67" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BD67" t="inlineStr">
         <is>
           <t>REGULAR</t>
         </is>
       </c>
-      <c r="BE63" t="inlineStr">
-        <is>
-          <t>19295</t>
-        </is>
-      </c>
-      <c r="BF63" t="inlineStr">
-        <is>
-          <t>263081,264584</t>
-        </is>
-      </c>
-      <c r="BG63" t="inlineStr">
-        <is>
-          <t>2037,2044</t>
-        </is>
-      </c>
-      <c r="BH63" t="inlineStr">
-        <is>
-          <t>eleven thousand two hundred fifty</t>
-        </is>
-      </c>
-      <c r="BI63" t="inlineStr">
-        <is>
-          <t>15599</t>
-        </is>
-      </c>
-      <c r="BJ63" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="BK63" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="BL63" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="BM63" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="BN63" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="BO63" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="BP63" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="BQ63" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="BR63" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="BS63" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="BT63" t="inlineStr">
+      <c r="BE67" t="inlineStr">
+        <is>
+          <t>18766</t>
+        </is>
+      </c>
+      <c r="BF67" t="inlineStr">
+        <is>
+          <t>262401,264163</t>
+        </is>
+      </c>
+      <c r="BG67" t="inlineStr">
+        <is>
+          <t>2037,2042</t>
+        </is>
+      </c>
+      <c r="BH67" t="inlineStr">
+        <is>
+          <t>eight thousand eight hundred fifty</t>
+        </is>
+      </c>
+      <c r="BI67" t="inlineStr">
+        <is>
+          <t>15541</t>
+        </is>
+      </c>
+      <c r="BJ67" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BK67" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BL67" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BM67" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BN67" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BO67" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BP67" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BQ67" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BR67" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BS67" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BT67" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="BU63" t="inlineStr">
+      <c r="BU67" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
-      <c r="BV63" t="inlineStr">
+      <c r="BV67" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>753702</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>1234</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>11000316759740</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>1763183095</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>8550.00</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>15-Nov-2025 10:35:50</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="M68" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="N68" t="inlineStr">
+        <is>
+          <t>108574613225</t>
+        </is>
+      </c>
+      <c r="O68" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P68" t="inlineStr">
+        <is>
+          <t>100000036600</t>
+        </is>
+      </c>
+      <c r="Q68" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="R68" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="S68" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="T68" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="U68" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="V68" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="W68" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="X68" t="inlineStr">
+        <is>
+          <t>DUVVU MAHALAKSHMI</t>
+        </is>
+      </c>
+      <c r="Y68" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="Z68" t="inlineStr">
+        <is>
+          <t>9502247535</t>
+        </is>
+      </c>
+      <c r="AA68" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AB68" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AC68" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AD68" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AE68" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AF68" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AG68" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AH68" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AI68" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="AJ68" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="AK68" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AL68" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AM68" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AN68" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AO68" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AP68" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AQ68" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AR68" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AS68" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AT68" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="AU68" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AV68" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AW68" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AX68" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AY68" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AZ68" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BA68" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="BB68" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="BC68" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BD68" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="BE68" t="inlineStr">
+        <is>
+          <t>18522</t>
+        </is>
+      </c>
+      <c r="BF68" t="inlineStr">
+        <is>
+          <t>262132,263952</t>
+        </is>
+      </c>
+      <c r="BG68" t="inlineStr">
+        <is>
+          <t>2037,2041</t>
+        </is>
+      </c>
+      <c r="BH68" t="inlineStr">
+        <is>
+          <t>eight thousand five hundred fifty</t>
+        </is>
+      </c>
+      <c r="BI68" t="inlineStr">
+        <is>
+          <t>16020</t>
+        </is>
+      </c>
+      <c r="BJ68" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BK68" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BL68" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BM68" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BN68" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BO68" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BP68" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BQ68" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BR68" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BS68" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BT68" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="BU68" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BV68" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>753702</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>1234</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>11000316792543</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>1763195595</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>8050.00</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>15-Nov-2025 14:02:46</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="M69" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="N69" t="inlineStr">
+        <is>
+          <t>689600444274</t>
+        </is>
+      </c>
+      <c r="O69" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P69" t="inlineStr">
+        <is>
+          <t>100000036600</t>
+        </is>
+      </c>
+      <c r="Q69" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="R69" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="S69" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="T69" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="U69" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="V69" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="W69" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="X69" t="inlineStr">
+        <is>
+          <t>MOHAMMAD ALINA SAMDANI</t>
+        </is>
+      </c>
+      <c r="Y69" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="Z69" t="inlineStr">
+        <is>
+          <t>8790615241</t>
+        </is>
+      </c>
+      <c r="AA69" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AB69" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AC69" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AD69" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AE69" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AF69" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AG69" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AH69" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AI69" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="AJ69" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="AK69" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AL69" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AM69" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AN69" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AO69" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AP69" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AQ69" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AR69" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AS69" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AT69" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="AU69" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AV69" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AW69" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AX69" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AY69" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AZ69" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BA69" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="BB69" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="BC69" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BD69" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="BE69" t="inlineStr">
+        <is>
+          <t>18523</t>
+        </is>
+      </c>
+      <c r="BF69" t="inlineStr">
+        <is>
+          <t>265622</t>
+        </is>
+      </c>
+      <c r="BG69" t="inlineStr">
+        <is>
+          <t>2049</t>
+        </is>
+      </c>
+      <c r="BH69" t="inlineStr">
+        <is>
+          <t>eight thousand fifty</t>
+        </is>
+      </c>
+      <c r="BI69" t="inlineStr">
+        <is>
+          <t>16795</t>
+        </is>
+      </c>
+      <c r="BJ69" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BK69" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BL69" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BM69" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BN69" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BO69" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+      <c r="BP69" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BQ69" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BR69" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BS69" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BT69" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="BU69" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BV69" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>753702</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>1234</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>11000316794728</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>1763196672</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>7750.00</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>15-Nov-2025 14:21:46</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="M70" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="N70" t="inlineStr">
+        <is>
+          <t>108575833074</t>
+        </is>
+      </c>
+      <c r="O70" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P70" t="inlineStr">
+        <is>
+          <t>100000036600</t>
+        </is>
+      </c>
+      <c r="Q70" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="R70" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="S70" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="T70" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="U70" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="V70" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="W70" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="X70" t="inlineStr">
+        <is>
+          <t>GUNIPE NIHARIKA</t>
+        </is>
+      </c>
+      <c r="Y70" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="Z70" t="inlineStr">
+        <is>
+          <t>9966262514</t>
+        </is>
+      </c>
+      <c r="AA70" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AB70" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AC70" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AD70" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AE70" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AF70" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AG70" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AH70" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AI70" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="AJ70" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="AK70" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AL70" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AM70" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AN70" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AO70" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AP70" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AQ70" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AR70" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AS70" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AT70" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="AU70" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AV70" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AW70" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AX70" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AY70" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AZ70" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BA70" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="BB70" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="BC70" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BD70" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="BE70" t="inlineStr">
+        <is>
+          <t>19893</t>
+        </is>
+      </c>
+      <c r="BF70" t="inlineStr">
+        <is>
+          <t>265185</t>
+        </is>
+      </c>
+      <c r="BG70" t="inlineStr">
+        <is>
+          <t>2048</t>
+        </is>
+      </c>
+      <c r="BH70" t="inlineStr">
+        <is>
+          <t>seven thousand seven hundred fifty</t>
+        </is>
+      </c>
+      <c r="BI70" t="inlineStr">
+        <is>
+          <t>17178</t>
+        </is>
+      </c>
+      <c r="BJ70" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BK70" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BL70" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BM70" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BN70" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BO70" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BP70" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BQ70" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BR70" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BS70" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BT70" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="BU70" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BV70" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>753702</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>1234</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>11000316837646</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>1763216495</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>8850.00</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>15-Nov-2025 19:52:03</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="K71" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="L71" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="M71" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="N71" t="inlineStr">
+        <is>
+          <t>108577731862</t>
+        </is>
+      </c>
+      <c r="O71" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P71" t="inlineStr">
+        <is>
+          <t>100000036600</t>
+        </is>
+      </c>
+      <c r="Q71" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="R71" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="S71" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="T71" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="U71" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="V71" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="W71" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="X71" t="inlineStr">
+        <is>
+          <t>KURAKULA JATHIN</t>
+        </is>
+      </c>
+      <c r="Y71" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="Z71" t="inlineStr">
+        <is>
+          <t>8106938482</t>
+        </is>
+      </c>
+      <c r="AA71" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AB71" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AC71" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AD71" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AE71" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AF71" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AG71" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AH71" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AI71" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="AJ71" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="AK71" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AL71" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AM71" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AN71" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AO71" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AP71" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AQ71" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AR71" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AS71" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AT71" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="AU71" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AV71" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AW71" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AX71" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AY71" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AZ71" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BA71" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="BB71" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="BC71" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BD71" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="BE71" t="inlineStr">
+        <is>
+          <t>18704</t>
+        </is>
+      </c>
+      <c r="BF71" t="inlineStr">
+        <is>
+          <t>262588,264203</t>
+        </is>
+      </c>
+      <c r="BG71" t="inlineStr">
+        <is>
+          <t>2037,2042</t>
+        </is>
+      </c>
+      <c r="BH71" t="inlineStr">
+        <is>
+          <t>eight thousand eight hundred fifty</t>
+        </is>
+      </c>
+      <c r="BI71" t="inlineStr">
+        <is>
+          <t>15915</t>
+        </is>
+      </c>
+      <c r="BJ71" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BK71" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BL71" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BM71" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BN71" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BO71" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BP71" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BQ71" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BR71" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BS71" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BT71" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="BU71" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BV71" t="inlineStr">
         <is>
           <t>-</t>
         </is>

</xml_diff>

<commit_message>
Update fee collection and transaction reports
Added new fee payment records and updated fee status for multiple students in CSV and Excel reports. Adjusted 'Total_Fee_Paid' and 'Total_Due' fields in fees_collection.csv to reflect recent payments. Updated transaction logs in fee_transcation_atom_report.csv and appended new entries to daywise and 2025-26 collection reports. Binary report and dashboard files were also updated to include the latest data.
</commit_message>
<xml_diff>
--- a/output_data/atom_report.xlsx
+++ b/output_data/atom_report.xlsx
@@ -24754,7 +24754,7 @@
       </c>
       <c r="M67" t="inlineStr">
         <is>
-          <t>NRNS</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="N67" t="inlineStr">
@@ -24779,7 +24779,7 @@
       </c>
       <c r="R67" t="inlineStr">
         <is>
-          <t/>
+          <t>17-Nov-2025 00:00:00</t>
         </is>
       </c>
       <c r="S67" t="inlineStr">
@@ -24854,12 +24854,12 @@
       </c>
       <c r="AG67" t="inlineStr">
         <is>
-          <t/>
+          <t>5</t>
         </is>
       </c>
       <c r="AH67" t="inlineStr">
         <is>
-          <t/>
+          <t>0.9</t>
         </is>
       </c>
       <c r="AI67" t="inlineStr">
@@ -24874,17 +24874,17 @@
       </c>
       <c r="AK67" t="inlineStr">
         <is>
-          <t/>
+          <t>5.9</t>
         </is>
       </c>
       <c r="AL67" t="inlineStr">
         <is>
-          <t/>
+          <t>8850.0</t>
         </is>
       </c>
       <c r="AM67" t="inlineStr">
         <is>
-          <t/>
+          <t>17-Nov-2025 00:00:00</t>
         </is>
       </c>
       <c r="AN67" t="inlineStr">
@@ -25126,7 +25126,7 @@
       </c>
       <c r="M68" t="inlineStr">
         <is>
-          <t>NRNS</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="N68" t="inlineStr">
@@ -25151,7 +25151,7 @@
       </c>
       <c r="R68" t="inlineStr">
         <is>
-          <t/>
+          <t>17-Nov-2025 00:00:00</t>
         </is>
       </c>
       <c r="S68" t="inlineStr">
@@ -25226,12 +25226,12 @@
       </c>
       <c r="AG68" t="inlineStr">
         <is>
-          <t/>
+          <t>5</t>
         </is>
       </c>
       <c r="AH68" t="inlineStr">
         <is>
-          <t/>
+          <t>0.9</t>
         </is>
       </c>
       <c r="AI68" t="inlineStr">
@@ -25246,17 +25246,17 @@
       </c>
       <c r="AK68" t="inlineStr">
         <is>
-          <t/>
+          <t>5.9</t>
         </is>
       </c>
       <c r="AL68" t="inlineStr">
         <is>
-          <t/>
+          <t>8550.0</t>
         </is>
       </c>
       <c r="AM68" t="inlineStr">
         <is>
-          <t/>
+          <t>17-Nov-2025 00:00:00</t>
         </is>
       </c>
       <c r="AN68" t="inlineStr">
@@ -25498,7 +25498,7 @@
       </c>
       <c r="M69" t="inlineStr">
         <is>
-          <t>NRNS</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="N69" t="inlineStr">
@@ -25523,7 +25523,7 @@
       </c>
       <c r="R69" t="inlineStr">
         <is>
-          <t/>
+          <t>17-Nov-2025 00:00:00</t>
         </is>
       </c>
       <c r="S69" t="inlineStr">
@@ -25598,12 +25598,12 @@
       </c>
       <c r="AG69" t="inlineStr">
         <is>
-          <t/>
+          <t>5</t>
         </is>
       </c>
       <c r="AH69" t="inlineStr">
         <is>
-          <t/>
+          <t>0.9</t>
         </is>
       </c>
       <c r="AI69" t="inlineStr">
@@ -25618,17 +25618,17 @@
       </c>
       <c r="AK69" t="inlineStr">
         <is>
-          <t/>
+          <t>5.9</t>
         </is>
       </c>
       <c r="AL69" t="inlineStr">
         <is>
-          <t/>
+          <t>8050.0</t>
         </is>
       </c>
       <c r="AM69" t="inlineStr">
         <is>
-          <t/>
+          <t>17-Nov-2025 00:00:00</t>
         </is>
       </c>
       <c r="AN69" t="inlineStr">
@@ -25870,7 +25870,7 @@
       </c>
       <c r="M70" t="inlineStr">
         <is>
-          <t>NRNS</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="N70" t="inlineStr">
@@ -25895,7 +25895,7 @@
       </c>
       <c r="R70" t="inlineStr">
         <is>
-          <t/>
+          <t>17-Nov-2025 00:00:00</t>
         </is>
       </c>
       <c r="S70" t="inlineStr">
@@ -25970,12 +25970,12 @@
       </c>
       <c r="AG70" t="inlineStr">
         <is>
-          <t/>
+          <t>5</t>
         </is>
       </c>
       <c r="AH70" t="inlineStr">
         <is>
-          <t/>
+          <t>0.9</t>
         </is>
       </c>
       <c r="AI70" t="inlineStr">
@@ -25990,17 +25990,17 @@
       </c>
       <c r="AK70" t="inlineStr">
         <is>
-          <t/>
+          <t>5.9</t>
         </is>
       </c>
       <c r="AL70" t="inlineStr">
         <is>
-          <t/>
+          <t>7750.0</t>
         </is>
       </c>
       <c r="AM70" t="inlineStr">
         <is>
-          <t/>
+          <t>17-Nov-2025 00:00:00</t>
         </is>
       </c>
       <c r="AN70" t="inlineStr">
@@ -26242,310 +26242,1798 @@
       </c>
       <c r="M71" t="inlineStr">
         <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="N71" t="inlineStr">
+        <is>
+          <t>108577731862</t>
+        </is>
+      </c>
+      <c r="O71" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P71" t="inlineStr">
+        <is>
+          <t>100000036600</t>
+        </is>
+      </c>
+      <c r="Q71" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="R71" t="inlineStr">
+        <is>
+          <t>17-Nov-2025 00:00:00</t>
+        </is>
+      </c>
+      <c r="S71" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="T71" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="U71" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="V71" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="W71" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="X71" t="inlineStr">
+        <is>
+          <t>KURAKULA JATHIN</t>
+        </is>
+      </c>
+      <c r="Y71" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="Z71" t="inlineStr">
+        <is>
+          <t>8106938482</t>
+        </is>
+      </c>
+      <c r="AA71" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AB71" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AC71" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AD71" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AE71" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AF71" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AG71" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AH71" t="inlineStr">
+        <is>
+          <t>0.9</t>
+        </is>
+      </c>
+      <c r="AI71" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="AJ71" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="AK71" t="inlineStr">
+        <is>
+          <t>5.9</t>
+        </is>
+      </c>
+      <c r="AL71" t="inlineStr">
+        <is>
+          <t>8850.0</t>
+        </is>
+      </c>
+      <c r="AM71" t="inlineStr">
+        <is>
+          <t>17-Nov-2025 00:00:00</t>
+        </is>
+      </c>
+      <c r="AN71" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AO71" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AP71" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AQ71" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AR71" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AS71" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AT71" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="AU71" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AV71" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AW71" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AX71" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AY71" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AZ71" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BA71" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="BB71" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="BC71" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BD71" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="BE71" t="inlineStr">
+        <is>
+          <t>18704</t>
+        </is>
+      </c>
+      <c r="BF71" t="inlineStr">
+        <is>
+          <t>262588,264203</t>
+        </is>
+      </c>
+      <c r="BG71" t="inlineStr">
+        <is>
+          <t>2037,2042</t>
+        </is>
+      </c>
+      <c r="BH71" t="inlineStr">
+        <is>
+          <t>eight thousand eight hundred fifty</t>
+        </is>
+      </c>
+      <c r="BI71" t="inlineStr">
+        <is>
+          <t>15915</t>
+        </is>
+      </c>
+      <c r="BJ71" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BK71" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BL71" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BM71" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BN71" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BO71" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BP71" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BQ71" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BR71" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BS71" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BT71" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="BU71" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BV71" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>753702</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>1234</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>11000317106839</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>1763373817</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>8850.00</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>17-Nov-2025 15:34:07</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="L72" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="M72" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="N72" t="inlineStr">
+        <is>
+          <t>253874637302</t>
+        </is>
+      </c>
+      <c r="O72" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P72" t="inlineStr">
+        <is>
+          <t>100000036600</t>
+        </is>
+      </c>
+      <c r="Q72" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="R72" t="inlineStr">
+        <is>
+          <t>18-Nov-2025 00:00:00</t>
+        </is>
+      </c>
+      <c r="S72" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="T72" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="U72" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="V72" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="W72" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="X72" t="inlineStr">
+        <is>
+          <t>GUNTURU VIDYA SRI</t>
+        </is>
+      </c>
+      <c r="Y72" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="Z72" t="inlineStr">
+        <is>
+          <t>8885883431</t>
+        </is>
+      </c>
+      <c r="AA72" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AB72" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AC72" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AD72" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AE72" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AF72" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AG72" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AH72" t="inlineStr">
+        <is>
+          <t>0.9</t>
+        </is>
+      </c>
+      <c r="AI72" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="AJ72" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="AK72" t="inlineStr">
+        <is>
+          <t>5.9</t>
+        </is>
+      </c>
+      <c r="AL72" t="inlineStr">
+        <is>
+          <t>8850.0</t>
+        </is>
+      </c>
+      <c r="AM72" t="inlineStr">
+        <is>
+          <t>18-Nov-2025 00:00:00</t>
+        </is>
+      </c>
+      <c r="AN72" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AO72" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AP72" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AQ72" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AR72" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AS72" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AT72" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="AU72" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AV72" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AW72" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AX72" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AY72" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AZ72" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BA72" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="BB72" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="BC72" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BD72" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="BE72" t="inlineStr">
+        <is>
+          <t>18960</t>
+        </is>
+      </c>
+      <c r="BF72" t="inlineStr">
+        <is>
+          <t>262774,264277</t>
+        </is>
+      </c>
+      <c r="BG72" t="inlineStr">
+        <is>
+          <t>2037,2042</t>
+        </is>
+      </c>
+      <c r="BH72" t="inlineStr">
+        <is>
+          <t>eight thousand eight hundred fifty</t>
+        </is>
+      </c>
+      <c r="BI72" t="inlineStr">
+        <is>
+          <t>17069</t>
+        </is>
+      </c>
+      <c r="BJ72" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BK72" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BL72" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BM72" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BN72" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BO72" t="inlineStr">
+        <is>
+          <t>UPI INTENT</t>
+        </is>
+      </c>
+      <c r="BP72" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BQ72" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BR72" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BS72" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BT72" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="BU72" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BV72" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>753702</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>1234</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>11000317244031</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>1763441830</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>11350.00</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>18-Nov-2025 10:28:43</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>VlllX</t>
+        </is>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="L73" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="M73" t="inlineStr">
+        <is>
           <t>NRNS</t>
         </is>
       </c>
-      <c r="N71" t="inlineStr">
-        <is>
-          <t>108577731862</t>
-        </is>
-      </c>
-      <c r="O71" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="P71" t="inlineStr">
+      <c r="N73" t="inlineStr">
+        <is>
+          <t>108591365446</t>
+        </is>
+      </c>
+      <c r="O73" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P73" t="inlineStr">
         <is>
           <t>100000036600</t>
         </is>
       </c>
-      <c r="Q71" t="inlineStr">
+      <c r="Q73" t="inlineStr">
         <is>
           <t>SIBL0000899</t>
         </is>
       </c>
-      <c r="R71" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="S71" t="inlineStr">
+      <c r="R73" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="S73" t="inlineStr">
         <is>
           <t>MERCHANT</t>
         </is>
       </c>
-      <c r="T71" t="inlineStr">
+      <c r="T73" t="inlineStr">
         <is>
           <t>UPI</t>
         </is>
       </c>
-      <c r="U71" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="V71" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="W71" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="X71" t="inlineStr">
-        <is>
-          <t>KURAKULA JATHIN</t>
-        </is>
-      </c>
-      <c r="Y71" t="inlineStr">
+      <c r="U73" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="V73" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="W73" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="X73" t="inlineStr">
+        <is>
+          <t>KONDALA JOSHNA</t>
+        </is>
+      </c>
+      <c r="Y73" t="inlineStr">
         <is>
           <t>kotakschoolvsp@gmail.com</t>
         </is>
       </c>
-      <c r="Z71" t="inlineStr">
-        <is>
-          <t>8106938482</t>
-        </is>
-      </c>
-      <c r="AA71" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="AB71" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="AC71" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="AD71" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="AE71" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="AF71" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="AG71" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="AH71" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="AI71" t="inlineStr">
+      <c r="Z73" t="inlineStr">
+        <is>
+          <t>8143411492</t>
+        </is>
+      </c>
+      <c r="AA73" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AB73" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AC73" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AD73" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AE73" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AF73" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AG73" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AH73" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AI73" t="inlineStr">
         <is>
           <t>0.00</t>
         </is>
       </c>
-      <c r="AJ71" t="inlineStr">
+      <c r="AJ73" t="inlineStr">
         <is>
           <t>0.00</t>
         </is>
       </c>
-      <c r="AK71" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="AL71" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="AM71" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="AN71" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="AO71" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="AP71" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="AQ71" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="AR71" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="AS71" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="AT71" t="inlineStr">
+      <c r="AK73" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AL73" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AM73" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AN73" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AO73" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AP73" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AQ73" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AR73" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AS73" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AT73" t="inlineStr">
         <is>
           <t>TRANSACTION IS SUCCESSFUL</t>
         </is>
       </c>
-      <c r="AU71" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="AV71" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="AW71" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="AX71" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="AY71" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="AZ71" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="BA71" t="inlineStr">
+      <c r="AU73" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AV73" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AW73" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AX73" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AY73" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AZ73" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BA73" t="inlineStr">
         <is>
           <t>UPI</t>
         </is>
       </c>
-      <c r="BB71" t="inlineStr">
+      <c r="BB73" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN SECONDARY SCHOOL ICSE</t>
+        </is>
+      </c>
+      <c r="BC73" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BD73" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="BE73" t="inlineStr">
+        <is>
+          <t>19383</t>
+        </is>
+      </c>
+      <c r="BF73" t="inlineStr">
+        <is>
+          <t>266397</t>
+        </is>
+      </c>
+      <c r="BG73" t="inlineStr">
+        <is>
+          <t>2053</t>
+        </is>
+      </c>
+      <c r="BH73" t="inlineStr">
+        <is>
+          <t>eleven thousand three hundred fifty</t>
+        </is>
+      </c>
+      <c r="BI73" t="inlineStr">
+        <is>
+          <t>14546</t>
+        </is>
+      </c>
+      <c r="BJ73" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BK73" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BL73" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BM73" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BN73" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BO73" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BP73" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BQ73" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BR73" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BS73" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BT73" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="BU73" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BV73" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>753702</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>1234</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>11000317263208</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>1763446046</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>16700.00</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>18-Nov-2025 11:39:14</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="L74" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="M74" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="N74" t="inlineStr">
+        <is>
+          <t>108591734203</t>
+        </is>
+      </c>
+      <c r="O74" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P74" t="inlineStr">
+        <is>
+          <t>100000036600</t>
+        </is>
+      </c>
+      <c r="Q74" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="R74" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="S74" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="T74" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="U74" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="V74" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="W74" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="X74" t="inlineStr">
+        <is>
+          <t>AKKURADA ARADHYA</t>
+        </is>
+      </c>
+      <c r="Y74" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="Z74" t="inlineStr">
+        <is>
+          <t>8500847900</t>
+        </is>
+      </c>
+      <c r="AA74" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AB74" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AC74" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AD74" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AE74" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AF74" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AG74" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AH74" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AI74" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="AJ74" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="AK74" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AL74" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AM74" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AN74" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AO74" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AP74" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AQ74" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AR74" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AS74" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AT74" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="AU74" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AV74" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AW74" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AX74" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AY74" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AZ74" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BA74" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="BB74" t="inlineStr">
         <is>
           <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
         </is>
       </c>
-      <c r="BC71" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="BD71" t="inlineStr">
+      <c r="BC74" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BD74" t="inlineStr">
         <is>
           <t>REGULAR</t>
         </is>
       </c>
-      <c r="BE71" t="inlineStr">
-        <is>
-          <t>18704</t>
-        </is>
-      </c>
-      <c r="BF71" t="inlineStr">
-        <is>
-          <t>262588,264203</t>
-        </is>
-      </c>
-      <c r="BG71" t="inlineStr">
-        <is>
-          <t>2037,2042</t>
-        </is>
-      </c>
-      <c r="BH71" t="inlineStr">
-        <is>
-          <t>eight thousand eight hundred fifty</t>
-        </is>
-      </c>
-      <c r="BI71" t="inlineStr">
-        <is>
-          <t>15915</t>
-        </is>
-      </c>
-      <c r="BJ71" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="BK71" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="BL71" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="BM71" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="BN71" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="BO71" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="BP71" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="BQ71" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="BR71" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="BS71" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="BT71" t="inlineStr">
+      <c r="BE74" t="inlineStr">
+        <is>
+          <t>20090</t>
+        </is>
+      </c>
+      <c r="BF74" t="inlineStr">
+        <is>
+          <t>268489,268490</t>
+        </is>
+      </c>
+      <c r="BG74" t="inlineStr">
+        <is>
+          <t>2050,2058</t>
+        </is>
+      </c>
+      <c r="BH74" t="inlineStr">
+        <is>
+          <t>sixteen thousand seven hundred</t>
+        </is>
+      </c>
+      <c r="BI74" t="inlineStr">
+        <is>
+          <t>17371</t>
+        </is>
+      </c>
+      <c r="BJ74" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BK74" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BL74" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BM74" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BN74" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BO74" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BP74" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BQ74" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BR74" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BS74" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BT74" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="BU71" t="inlineStr">
+      <c r="BU74" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
-      <c r="BV71" t="inlineStr">
+      <c r="BV74" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>SALESIAN EDUCATION SOCIETY</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>753702</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>1234</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>11000317317733</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>1763464253</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>8350.00</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>18-Nov-2025 16:41:50</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>lVl</t>
+        </is>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>sale</t>
+        </is>
+      </c>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t>ICICI UPI QR</t>
+        </is>
+      </c>
+      <c r="L75" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="M75" t="inlineStr">
+        <is>
+          <t>NRNS</t>
+        </is>
+      </c>
+      <c r="N75" t="inlineStr">
+        <is>
+          <t>108593680409</t>
+        </is>
+      </c>
+      <c r="O75" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P75" t="inlineStr">
+        <is>
+          <t>100000036600</t>
+        </is>
+      </c>
+      <c r="Q75" t="inlineStr">
+        <is>
+          <t>SIBL0000899</t>
+        </is>
+      </c>
+      <c r="R75" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="S75" t="inlineStr">
+        <is>
+          <t>MERCHANT</t>
+        </is>
+      </c>
+      <c r="T75" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="U75" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="V75" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="W75" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="X75" t="inlineStr">
+        <is>
+          <t>VEDITHI ARPANA CHANDRA</t>
+        </is>
+      </c>
+      <c r="Y75" t="inlineStr">
+        <is>
+          <t>kotakschoolvsp@gmail.com</t>
+        </is>
+      </c>
+      <c r="Z75" t="inlineStr">
+        <is>
+          <t>9959307771</t>
+        </is>
+      </c>
+      <c r="AA75" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AB75" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AC75" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AD75" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AE75" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AF75" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AG75" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AH75" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AI75" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="AJ75" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="AK75" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AL75" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AM75" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AN75" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AO75" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AP75" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AQ75" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AR75" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AS75" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AT75" t="inlineStr">
+        <is>
+          <t>TRANSACTION IS SUCCESSFUL</t>
+        </is>
+      </c>
+      <c r="AU75" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AV75" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AW75" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AX75" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AY75" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AZ75" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BA75" t="inlineStr">
+        <is>
+          <t>UPI</t>
+        </is>
+      </c>
+      <c r="BB75" t="inlineStr">
+        <is>
+          <t>KOTAK SALESIAN PRIMARY SCHOOL</t>
+        </is>
+      </c>
+      <c r="BC75" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BD75" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="BE75" t="inlineStr">
+        <is>
+          <t>18863</t>
+        </is>
+      </c>
+      <c r="BF75" t="inlineStr">
+        <is>
+          <t>265936</t>
+        </is>
+      </c>
+      <c r="BG75" t="inlineStr">
+        <is>
+          <t>2050</t>
+        </is>
+      </c>
+      <c r="BH75" t="inlineStr">
+        <is>
+          <t>eight thousand three hundred fifty</t>
+        </is>
+      </c>
+      <c r="BI75" t="inlineStr">
+        <is>
+          <t>15938</t>
+        </is>
+      </c>
+      <c r="BJ75" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BK75" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BL75" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BM75" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BN75" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BO75" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BP75" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BQ75" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BR75" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BS75" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BT75" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="BU75" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="BV75" t="inlineStr">
         <is>
           <t>-</t>
         </is>

</xml_diff>